<commit_message>
remove redundant BUZZ pin from PA4
</commit_message>
<xml_diff>
--- a/design_documents/design.xlsx
+++ b/design_documents/design.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/74db7c87a9029f2a/Documents/PCB/SmallFlight1/design_documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="416" documentId="11_F25DC773A252ABDACC1048E409DB493A5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DDDECED4-F47D-49F5-B84B-89BE706D00E4}"/>
+  <xr:revisionPtr revIDLastSave="423" documentId="11_F25DC773A252ABDACC1048E409DB493A5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{506582A0-D5D9-4D12-A738-03E0602F8101}"/>
   <bookViews>
-    <workbookView xWindow="4200" yWindow="1860" windowWidth="21240" windowHeight="11415" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="26040" windowHeight="11970" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ideation" sheetId="1" r:id="rId1"/>
@@ -353,7 +353,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -370,16 +370,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -676,22 +670,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="E1" s="6" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="E1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
+      <c r="A2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
       <c r="E2" s="3" t="s">
         <v>8</v>
       </c>
@@ -706,9 +700,9 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
+      <c r="A3" s="7"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
       <c r="E3" s="2" t="s">
         <v>9</v>
       </c>
@@ -836,13 +830,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -874,7 +868,7 @@
       <c r="D3" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="5" t="s">
         <v>51</v>
       </c>
     </row>
@@ -891,7 +885,7 @@
       <c r="D4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="5" t="s">
         <v>43</v>
       </c>
     </row>
@@ -908,7 +902,7 @@
       <c r="D5" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="5" t="s">
         <v>64</v>
       </c>
     </row>
@@ -925,7 +919,7 @@
       <c r="D6" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="5" t="s">
         <v>58</v>
       </c>
     </row>
@@ -942,7 +936,7 @@
       <c r="D7" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="5" t="s">
         <v>46</v>
       </c>
     </row>
@@ -976,7 +970,7 @@
       <c r="D9" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="5" t="s">
         <v>53</v>
       </c>
     </row>
@@ -986,6 +980,12 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E8" r:id="rId1" xr:uid="{29E36415-BC89-409B-9AAB-729EDB483B27}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{52B35B77-BA62-4550-BBBC-BF68DD70E8AF}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{7656E701-F02C-4FF5-BE5A-0ADB400D8BCD}"/>
+    <hyperlink ref="E5" r:id="rId4" xr:uid="{87BD5190-CE07-49F7-B8B4-308BFC6B4F76}"/>
+    <hyperlink ref="E6" r:id="rId5" xr:uid="{5391E0E2-5DD2-4B74-80CF-DF358EDFFAFF}"/>
+    <hyperlink ref="E7" r:id="rId6" xr:uid="{51AE9F35-F79A-4530-B051-D14B2B71A81F}"/>
+    <hyperlink ref="E9" r:id="rId7" xr:uid="{34D1A06B-5E40-4E9F-B6F9-65DE6507D8D2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1006,40 +1006,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7" t="s">
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="I2" s="9" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="I2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="K2" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="L2" s="3" t="s">
         <v>78</v>
       </c>
       <c r="M2" s="3" t="s">
@@ -1047,7 +1047,7 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="7"/>
+      <c r="A3" s="6"/>
       <c r="B3" s="3" t="s">
         <v>65</v>
       </c>
@@ -1066,16 +1066,16 @@
       <c r="G3" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="J3" s="8">
+      <c r="J3" s="2">
         <v>3.7</v>
       </c>
-      <c r="K3" s="8">
+      <c r="K3" s="2">
         <v>400</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="2">
         <v>1</v>
       </c>
       <c r="M3" s="2" t="s">
@@ -1104,16 +1104,16 @@
       <c r="G4" s="2">
         <v>240</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="J4" s="8">
+      <c r="J4" s="2">
         <v>3.7</v>
       </c>
-      <c r="K4" s="8">
+      <c r="K4" s="2">
         <v>1100</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="2">
         <v>2</v>
       </c>
       <c r="M4" s="2" t="s">

</xml_diff>